<commit_message>
Falta detallar los reportes y probarlos del todo
</commit_message>
<xml_diff>
--- a/actividades.xlsx
+++ b/actividades.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L2"/>
+  <dimension ref="A1:L3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -545,6 +545,66 @@
         </is>
       </c>
       <c r="L2" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Realizar seguimiento a solicitudes y requerimientos tecnológicos de los usuarios, documentando novedades, avances y necesidades adicionales, y comunicándolas oportunamente a los responsables correspondientes.</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>2026-02-13 12:00:22</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>COMUNICACIONES</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Valentina</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>APOYO TECNOLÓGICO</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>LLAMADA TELEFONICA</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>Se solicita la revisión de un problema con la aplicación de lectura de los archivos, se hace la revisión correspondiente y se instala una aplicación de lectura de archivos diferente al solicitante, se le informa al solicitante sobre esto</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>2026-02-20</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>Se solicita la revisión de un problema con la aplicación de lectura de los archivos, se hace la revisión correspondiente y se instala una aplicación de lectura de archivos diferente al solicitante, se le informa al solicitante sobre esto</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
         <is>
           <t>admin</t>
         </is>

</xml_diff>

<commit_message>
Actualizado e instalado en local
</commit_message>
<xml_diff>
--- a/actividades.xlsx
+++ b/actividades.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K44"/>
+  <dimension ref="A1:K64"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1641,7 +1641,7 @@
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>APOYO TECNOLÓGICO</t>
+          <t>Configuración</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
@@ -1661,7 +1661,7 @@
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>2026-03-23</t>
+          <t>2026-03-24</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
@@ -2921,6 +2921,1146 @@
       <c r="K44" t="inlineStr">
         <is>
           <t>Se solicita la revisión de un email sospechoso, se revisa correspondientemente los datos y los links de dicho Email y se concluye que es un correo malicioso se procede a bloquear dicho correo desde donde se envió y se le informa a la solicitante</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>Alejandro</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>5.	Realizar seguimiento a solicitudes y requerimientos tecnológicos de los usuarios, documentando novedades, avances y necesidades adicionales, y comunicándolas oportunamente a los responsables correspondientes.</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>2026-04-08 11:09:27</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>CONTABILIDAD</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>Erica Marin</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>Software</t>
+        </is>
+      </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>E-MAIL</t>
+        </is>
+      </c>
+      <c r="H45" t="inlineStr">
+        <is>
+          <t>Se solicita la asignacion de permisos requeridos, se hace la asignacion de permisos requeridos y se le informa a la solicitante</t>
+        </is>
+      </c>
+      <c r="I45" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="J45" t="inlineStr">
+        <is>
+          <t>2026-04-08</t>
+        </is>
+      </c>
+      <c r="K45" t="inlineStr">
+        <is>
+          <t>Se solicita la asignacion de permisos requeridos, se hace la asignacion de permisos requeridos y se le informa a la solicitante</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>Alejandro</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>5.	Realizar seguimiento a solicitudes y requerimientos tecnológicos de los usuarios, documentando novedades, avances y necesidades adicionales, y comunicándolas oportunamente a los responsables correspondientes.</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>2026-04-08 11:11:31</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>HACIENDA</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>Yuliana Ruiz Jaramillo</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>Software</t>
+        </is>
+      </c>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>E-MAIL</t>
+        </is>
+      </c>
+      <c r="H46" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Se solicita la creación de un nuevo usuario para un nuevo contratista, se hace la solicitud respectiva a la mesa de Saimyr y se le informa el usuario a la solicitante </t>
+        </is>
+      </c>
+      <c r="I46" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="J46" t="inlineStr">
+        <is>
+          <t>2026-04-08</t>
+        </is>
+      </c>
+      <c r="K46" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Se solicita la creación de un nuevo usuario para un nuevo contratista, se hace la solicitud respectiva a la mesa de Saimyr y se le informa el usuario a la solicitante </t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>Alejandro</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>6.	Apoyar en la documentación técnica del área, incluyendo la organización y archivo de documentos, informes de soporte y demás registros, de acuerdo con las directrices internas y del Sistema de Gestión de Calidad.</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>2026-04-09 11:12:40</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>HACIENDA</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>Yuliana Ruiz Jaramillo</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>Software</t>
+        </is>
+      </c>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>E-MAIL</t>
+        </is>
+      </c>
+      <c r="H47" t="inlineStr">
+        <is>
+          <t>Se solicita la asignación de permisos a un usuario, se hace la asignación de permisos requerida y se le informa a la solicitante</t>
+        </is>
+      </c>
+      <c r="I47" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="J47" t="inlineStr">
+        <is>
+          <t>2026-04-09</t>
+        </is>
+      </c>
+      <c r="K47" t="inlineStr">
+        <is>
+          <t>Se solicita la asignación de permisos a un usuario, se hace la asignación de permisos requerida y se le informa a la solicitante</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>Alejandro</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>5.	Realizar seguimiento a solicitudes y requerimientos tecnológicos de los usuarios, documentando novedades, avances y necesidades adicionales, y comunicándolas oportunamente a los responsables correspondientes.</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>2026-04-09 11:14:33</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>TESORERIA</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>Steven</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>Software</t>
+        </is>
+      </c>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>E-MAIL</t>
+        </is>
+      </c>
+      <c r="H48" t="inlineStr">
+        <is>
+          <t>Se solicita la creación de un usuario y los permisos respectivos a este, se hace la solicitud y se asignan los permisos requerido, se le informa al solicitante la información respectiva</t>
+        </is>
+      </c>
+      <c r="I48" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="J48" t="inlineStr">
+        <is>
+          <t>2026-04-09</t>
+        </is>
+      </c>
+      <c r="K48" t="inlineStr">
+        <is>
+          <t>Se solicita la creación de un usuario y los permisos respectivos a este, se hace la solicitud y se asignan los permisos requerido, se le informa al solicitante la información respectiva</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>Alejandro</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>5.	Realizar seguimiento a solicitudes y requerimientos tecnológicos de los usuarios, documentando novedades, avances y necesidades adicionales, y comunicándolas oportunamente a los responsables correspondientes.</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>2026-04-10 11:20:03</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>ALMACEN MUNICIPAL</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>Claudia Marcela Álvarez Chica</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>Software</t>
+        </is>
+      </c>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>E-MAIL</t>
+        </is>
+      </c>
+      <c r="H49" t="inlineStr">
+        <is>
+          <t>Se solicita cambio de contraseña para el acceso a los modulo, se hace el cambio respectivo y se le informa a la solicitante</t>
+        </is>
+      </c>
+      <c r="I49" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="J49" t="inlineStr">
+        <is>
+          <t>2026-04-10</t>
+        </is>
+      </c>
+      <c r="K49" t="inlineStr">
+        <is>
+          <t>Se solicita cambio de contraseña para el acceso a los modulo, se hace el cambio respectivo y se le informa a la solicitante</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>Alejandro</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>5.	Realizar seguimiento a solicitudes y requerimientos tecnológicos de los usuarios, documentando novedades, avances y necesidades adicionales, y comunicándolas oportunamente a los responsables correspondientes.</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>2026-04-10 11:32:20</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>HACIENDA</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>Lina Maria Rios</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>Software</t>
+        </is>
+      </c>
+      <c r="G50" t="inlineStr">
+        <is>
+          <t>E-MAIL</t>
+        </is>
+      </c>
+      <c r="H50" t="inlineStr">
+        <is>
+          <t>Se solicita el cambio de contraseña para el acceso del usuario a los módulos, se hace el cambio de contraseña respectivo y se le deja evidenciado a la solicitante el funcionamiento de este</t>
+        </is>
+      </c>
+      <c r="I50" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="J50" t="inlineStr">
+        <is>
+          <t>2026-04-10</t>
+        </is>
+      </c>
+      <c r="K50" t="inlineStr">
+        <is>
+          <t>Se solicita el cambio de contraseña para el acceso del usuario a los módulos, se hace el cambio de contraseña respectivo y se le deja evidenciado a la solicitante el funcionamiento de este</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>Alejandro</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>7.	Colaborar en la implementación y seguimiento de medidas básicas de seguridad informática, tales como el monitoreo de alertas básicas, cierre adecuado de sesiones, y cumplimiento de rutinas establecidas para el uso seguro de los recursos tecnológicos.</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>2026-04-10 11:46:11</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>FAMILIA</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>Luis Alejandro</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>Red/Conectividad</t>
+        </is>
+      </c>
+      <c r="G51" t="inlineStr">
+        <is>
+          <t>LLAMADA TELEFONICA</t>
+        </is>
+      </c>
+      <c r="H51" t="inlineStr">
+        <is>
+          <t>Se solicita el cambio de contraseña de ingreso al equipo de computo, se hace el cambio respectivo de acuerdo a los solicitado por el funcionario y se le deja evidenciado el normal funcionamiento</t>
+        </is>
+      </c>
+      <c r="I51" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="J51" t="inlineStr">
+        <is>
+          <t>2026-04-10</t>
+        </is>
+      </c>
+      <c r="K51" t="inlineStr">
+        <is>
+          <t>Se solicita el cambio de contraseña de ingreso al equipo de computo, se hace el cambio respectivo de acuerdo a los solicitado por el funcionario y se le deja evidenciado el normal funcionamiento</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>Alejandro</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>2.	Apoyar en el mantenimiento preventivo básico de equipos tecnológicos, realizando tareas como limpieza, revisión de cables, conectores y periféricos, con el objetivo de mantener en condiciones óptimas los recursos informáticos de la entidad.</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>2026-04-10 13:52:08</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>FAMILIA</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>Cristina</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>Software</t>
+        </is>
+      </c>
+      <c r="G52" t="inlineStr">
+        <is>
+          <t>VERBAL</t>
+        </is>
+      </c>
+      <c r="H52" t="inlineStr">
+        <is>
+          <t>Se solicita la instalación de un medio que pueda hacer copias de seguridad tiendo copia de seguridad del equipo y evitando perdida de archivos</t>
+        </is>
+      </c>
+      <c r="I52" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="J52" t="inlineStr">
+        <is>
+          <t>2026-04-10</t>
+        </is>
+      </c>
+      <c r="K52" t="inlineStr">
+        <is>
+          <t>Se solicita la instalación de un medio que pueda hacer copias de seguridad tiendo copia de seguridad del equipo y evitando perdida de archivos</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>Alejandro</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>5.	Realizar seguimiento a solicitudes y requerimientos tecnológicos de los usuarios, documentando novedades, avances y necesidades adicionales, y comunicándolas oportunamente a los responsables correspondientes.</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>2026-04-13 13:58:24</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>PLANEACIÓN</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>Manuela Garcia Arroyave</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>Software</t>
+        </is>
+      </c>
+      <c r="G53" t="inlineStr">
+        <is>
+          <t>E-MAIL</t>
+        </is>
+      </c>
+      <c r="H53" t="inlineStr">
+        <is>
+          <t>Se solicita la asignación de permisos para un usuario, se realiza la asignación de permisos solicitados y se le informa al solicitante</t>
+        </is>
+      </c>
+      <c r="I53" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="J53" t="inlineStr">
+        <is>
+          <t>2026-04-13</t>
+        </is>
+      </c>
+      <c r="K53" t="inlineStr">
+        <is>
+          <t>Se solicita la asignación de permisos para un usuario, se realiza la asignación de permisos solicitados y se le informa al solicitante</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>Alejandro</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>1.	Brindar apoyo en la atención de requerimientos técnicos de primer nivel a los usuarios de la Administración Municipal, atendiendo incidentes relacionados con el funcionamiento de equipos de cómputo, impresoras, configuración de software y otros periféricos.</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>2026-04-13 14:06:11</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>PLANEACIÓN</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>Juan Rodrigo Osorio Urrego  Técnico Operativo</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>Software</t>
+        </is>
+      </c>
+      <c r="G54" t="inlineStr">
+        <is>
+          <t>Email</t>
+        </is>
+      </c>
+      <c r="H54" t="inlineStr">
+        <is>
+          <t>Se solicita la asignación de permisos para un usuario, se hace la asignación de permisos respectivos y se le informa al solicitante</t>
+        </is>
+      </c>
+      <c r="I54" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="J54" t="inlineStr">
+        <is>
+          <t>2026-04-13</t>
+        </is>
+      </c>
+      <c r="K54" t="inlineStr">
+        <is>
+          <t>Se solicita la asignación de permisos para un usuario, se hace la asignación de permisos respectivos y se le informa al solicitante</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>Alejandro</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>7.	Colaborar en la implementación y seguimiento de medidas básicas de seguridad informática, tales como el monitoreo de alertas básicas, cierre adecuado de sesiones, y cumplimiento de rutinas establecidas para el uso seguro de los recursos tecnológicos.</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>2026-04-13 14:08:03</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>PROTECCION SOCIAL</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>Marleny Alzate Ocampo</t>
+        </is>
+      </c>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>Red/Conectividad</t>
+        </is>
+      </c>
+      <c r="G55" t="inlineStr">
+        <is>
+          <t>LLAMADA TELEFONICA</t>
+        </is>
+      </c>
+      <c r="H55" t="inlineStr">
+        <is>
+          <t>Se solicita cambio de contraseña para el equipo del solicitante, se hace el cambio y se le informa al solicitante</t>
+        </is>
+      </c>
+      <c r="I55" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="J55" t="inlineStr">
+        <is>
+          <t>2026-04-13</t>
+        </is>
+      </c>
+      <c r="K55" t="inlineStr">
+        <is>
+          <t>Se solicita cambio de contraseña para el equipo del solicitante, se hace el cambio y se le informa al solicitante</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>Alejandro</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>1.	Brindar apoyo en la atención de requerimientos técnicos de primer nivel a los usuarios de la Administración Municipal, atendiendo incidentes relacionados con el funcionamiento de equipos de cómputo, impresoras, configuración de software y otros periféricos.</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>2026-04-15 11:57:18</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>PLANEACIÓN</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>Estefania</t>
+        </is>
+      </c>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>Red/Conectividad</t>
+        </is>
+      </c>
+      <c r="G56" t="inlineStr">
+        <is>
+          <t>LLAMADA TELEFONICA</t>
+        </is>
+      </c>
+      <c r="H56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Se solicita la revision de la conexión del equipo de computo y el telefono que le proporciona la red de internet al equipo no se encontraba funcionando, a traves de una revision del cableado se hace una revision en el RAC y se desurbre que el cable estaba desconectado, se conecta el cable y vuelve a funcionar normalmente el equipo </t>
+        </is>
+      </c>
+      <c r="I56" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="J56" t="inlineStr">
+        <is>
+          <t>2026-04-15</t>
+        </is>
+      </c>
+      <c r="K56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Se solicita la revision de la conexión del equipo de computo y el telefono que le proporciona la red de internet al equipo no se encontraba funcionando, a traves de una revision del cableado se hace una revision en el RAC y se desurbre que el cable estaba desconectado, se conecta el cable y vuelve a funcionar normalmente el equipo </t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>Alejandro</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>5.	Realizar seguimiento a solicitudes y requerimientos tecnológicos de los usuarios, documentando novedades, avances y necesidades adicionales, y comunicándolas oportunamente a los responsables correspondientes.</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>2026-04-14 11:59:10</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>IMPUESTOS</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>Miguel Salazar</t>
+        </is>
+      </c>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>Software</t>
+        </is>
+      </c>
+      <c r="G57" t="inlineStr">
+        <is>
+          <t>E-MAIL</t>
+        </is>
+      </c>
+      <c r="H57" t="inlineStr">
+        <is>
+          <t>Se solicita la revision y el presente de una cuenta bloqueda de Saimyr, se hace la solicitud a la mesa de ayuda y resulven el caso, se informa y se evidencia con el funcionario afectado el correcto funcionamiento</t>
+        </is>
+      </c>
+      <c r="I57" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="J57" t="inlineStr">
+        <is>
+          <t>2026-04-14</t>
+        </is>
+      </c>
+      <c r="K57" t="inlineStr">
+        <is>
+          <t>Se solicita la revision y el presente de una cuenta bloqueda de Saimyr, se hace la solicitud a la mesa de ayuda y resulven el caso, se informa y se evidencia con el funcionario afectado el correcto funcionamiento</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>Alejandro</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>5.	Realizar seguimiento a solicitudes y requerimientos tecnológicos de los usuarios, documentando novedades, avances y necesidades adicionales, y comunicándolas oportunamente a los responsables correspondientes.</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>2026-04-14 12:01:42</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>IMPUESTOS</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>Elizabeth Tibaquira</t>
+        </is>
+      </c>
+      <c r="F58" t="inlineStr">
+        <is>
+          <t>Configuración</t>
+        </is>
+      </c>
+      <c r="G58" t="inlineStr">
+        <is>
+          <t>E-MAIL</t>
+        </is>
+      </c>
+      <c r="H58" t="inlineStr">
+        <is>
+          <t>Se solicita la asignacion de permisos para que el nuevo funcionario pueda apoyar mas en tema de impuestos, se hace la asignacion correspondiente de los permisos y se le informa a la solicitante</t>
+        </is>
+      </c>
+      <c r="I58" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="J58" t="inlineStr">
+        <is>
+          <t>2026-04-14</t>
+        </is>
+      </c>
+      <c r="K58" t="inlineStr">
+        <is>
+          <t>Se solicita la asignacion de permisos para que el nuevo funcionario pueda apoyar mas en tema de impuestos, se hace la asignacion correspondiente de los permisos y se le informa a la solicitante</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>Alejandro</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>7.	Colaborar en la implementación y seguimiento de medidas básicas de seguridad informática, tales como el monitoreo de alertas básicas, cierre adecuado de sesiones, y cumplimiento de rutinas establecidas para el uso seguro de los recursos tecnológicos.</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>2026-04-16 08:17:52</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>PROTECCION SOCIAL</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>Alejandro</t>
+        </is>
+      </c>
+      <c r="F59" t="inlineStr">
+        <is>
+          <t>Software</t>
+        </is>
+      </c>
+      <c r="G59" t="inlineStr">
+        <is>
+          <t>LLAMADA TELEFONICA</t>
+        </is>
+      </c>
+      <c r="H59" t="inlineStr">
+        <is>
+          <t>Se solicita cambio de contraseña del correo electronico para pode ingresar a el correo institucional, se hace el cambio de contraseña y se le evidencia al usuario el ingreso normal al correo electronico</t>
+        </is>
+      </c>
+      <c r="I59" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="J59" t="inlineStr">
+        <is>
+          <t>2026-04-16</t>
+        </is>
+      </c>
+      <c r="K59" t="inlineStr">
+        <is>
+          <t>Se solicita cambio de contraseña del correo electronico para pode ingresar a el correo institucional, se hace el cambio de contraseña y se le evidencia al usuario el ingreso normal al correo electronico</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>Alejandro</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>2.	Apoyar en el mantenimiento preventivo básico de equipos tecnológicos, realizando tareas como limpieza, revisión de cables, conectores y periféricos, con el objetivo de mantener en condiciones óptimas los recursos informáticos de la entidad.</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>2026-04-16 08:20:11</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>PLANEACIÓN</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>Angelica</t>
+        </is>
+      </c>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t>Red/Conectividad</t>
+        </is>
+      </c>
+      <c r="G60" t="inlineStr">
+        <is>
+          <t>LLAMADA TELEFONICA</t>
+        </is>
+      </c>
+      <c r="H60" t="inlineStr">
+        <is>
+          <t>Se solicita la revsion de la conectividad a Red de las caprtas compartidas, se hace la revision correspondiente y se le deja una ip fija, evidenciando que vuelven a funcionar normalmente las carpetas</t>
+        </is>
+      </c>
+      <c r="I60" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="J60" t="inlineStr">
+        <is>
+          <t>2026-04-16</t>
+        </is>
+      </c>
+      <c r="K60" t="inlineStr">
+        <is>
+          <t>Se solicita la revsion de la conectividad a Red de las caprtas compartidas, se hace la revision correspondiente y se le deja una ip fija, evidenciando que vuelven a funcionar normalmente las carpetas</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>Alejandro</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>2.	Apoyar en el mantenimiento preventivo básico de equipos tecnológicos, realizando tareas como limpieza, revisión de cables, conectores y periféricos, con el objetivo de mantener en condiciones óptimas los recursos informáticos de la entidad.</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>2026-04-16 08:23:15</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>PLANEACIÓN</t>
+        </is>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>Walter Dario</t>
+        </is>
+      </c>
+      <c r="F61" t="inlineStr">
+        <is>
+          <t>Red/Conectividad</t>
+        </is>
+      </c>
+      <c r="G61" t="inlineStr">
+        <is>
+          <t>LLAMADA TELEFONICA</t>
+        </is>
+      </c>
+      <c r="H61" t="inlineStr">
+        <is>
+          <t>Se solicita la conexion a las carpetas de red de la administración se le asigna al equipo una ip fija y se le evidencia al funcionario el correcto funcionamiento</t>
+        </is>
+      </c>
+      <c r="I61" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="J61" t="inlineStr">
+        <is>
+          <t>2026-04-16</t>
+        </is>
+      </c>
+      <c r="K61" t="inlineStr">
+        <is>
+          <t>Se solicita la conexion a las carpetas de red de la administración se le asigna al equipo una ip fija y se le evidencia al funcionario el correcto funcionamiento</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>Alejandro</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>1.	Brindar apoyo en la atención de requerimientos técnicos de primer nivel a los usuarios de la Administración Municipal, atendiendo incidentes relacionados con el funcionamiento de equipos de cómputo, impresoras, configuración de software y otros periféricos.</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>2026-04-16 08:23:53</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>PLANEACIÓN</t>
+        </is>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>Juan</t>
+        </is>
+      </c>
+      <c r="F62" t="inlineStr">
+        <is>
+          <t>Red/Conectividad</t>
+        </is>
+      </c>
+      <c r="G62" t="inlineStr">
+        <is>
+          <t>VERBAL</t>
+        </is>
+      </c>
+      <c r="H62" t="inlineStr">
+        <is>
+          <t>Se solicita la conexion a las carpetas de red de la administración se le asigna al equipo una ip fija y se le evidencia al funcionario el correcto funcionamiento</t>
+        </is>
+      </c>
+      <c r="I62" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="J62" t="inlineStr">
+        <is>
+          <t>2026-04-16</t>
+        </is>
+      </c>
+      <c r="K62" t="inlineStr">
+        <is>
+          <t>Se solicita la conexion a las carpetas de red de la administración se le asigna al equipo una ip fija y se le evidencia al funcionario el correcto funcionamiento</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>Alejandro</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>1.	Brindar apoyo en la atención de requerimientos técnicos de primer nivel a los usuarios de la Administración Municipal, atendiendo incidentes relacionados con el funcionamiento de equipos de cómputo, impresoras, configuración de software y otros periféricos.</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>2026-04-16 08:25:00</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>PLANEACIÓN</t>
+        </is>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>Angelica</t>
+        </is>
+      </c>
+      <c r="F63" t="inlineStr">
+        <is>
+          <t>Impresoras</t>
+        </is>
+      </c>
+      <c r="G63" t="inlineStr">
+        <is>
+          <t>VERBAL</t>
+        </is>
+      </c>
+      <c r="H63" t="inlineStr">
+        <is>
+          <t>Se solicita la revision de la conexion a la impresora, se hace la revision correspondiente y se le asigna una ip fija, se le evidencia el normal funcionamiento con la impresora y escaner</t>
+        </is>
+      </c>
+      <c r="I63" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="J63" t="inlineStr">
+        <is>
+          <t>2026-04-16</t>
+        </is>
+      </c>
+      <c r="K63" t="inlineStr">
+        <is>
+          <t>Se solicita la revision de la conexion a la impresora, se hace la revision correspondiente y se le asigna una ip fija, se le evidencia el normal funcionamiento con la impresora y escaner</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>Alejandro</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>1.	Brindar apoyo en la atención de requerimientos técnicos de primer nivel a los usuarios de la Administración Municipal, atendiendo incidentes relacionados con el funcionamiento de equipos de cómputo, impresoras, configuración de software y otros periféricos.</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>2026-04-16 09:07:19</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>PLANEACIÓN</t>
+        </is>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>Angelica</t>
+        </is>
+      </c>
+      <c r="F64" t="inlineStr">
+        <is>
+          <t>Impresoras</t>
+        </is>
+      </c>
+      <c r="G64" t="inlineStr">
+        <is>
+          <t>VERBAL</t>
+        </is>
+      </c>
+      <c r="H64" t="inlineStr">
+        <is>
+          <t>Se solicita la revsion de la impresora por un atasco de papel, se retira el atasco y se busca el motivo y se descubre que el fusor de la M636 se le despego el actato, se hace el cambio con un fusor de repuesto y se dejaevidenciado el normal funcionamiento</t>
+        </is>
+      </c>
+      <c r="I64" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="J64" t="inlineStr">
+        <is>
+          <t>2026-04-16</t>
+        </is>
+      </c>
+      <c r="K64" t="inlineStr">
+        <is>
+          <t>Se solicita la revsion de la impresora por un atasco de papel, se retira el atasco y se busca el motivo y se descubre que el fusor de la M636 se le despego el actato, se hace el cambio con un fusor de repuesto y se dejaevidenciado el normal funcionamiento</t>
         </is>
       </c>
     </row>

</xml_diff>